<commit_message>
Aquatic toxicity fatty acids, folpet and fluopicolide
For fatty acids, I invented the active substance name from
the old EU variant mentioning C7-C18 and C18 unsaturated to
"Fatty acids C10-C20, potassium salts" as it seems that smaller chain
lengths are not main components and the product from Alpha Biopesticides
made from olive oil ranges up to C20. I also defined the main components
listed in the draft RAR published 2023 as chemical entities, with the
help of PubChem, but the potassium salts of the more exotic acids do not
have PubChem entries.
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/fatty_acids_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/fatty_acids_aquatic_toxicity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDF171D-C1B7-4228-9F0F-EF7D5D1E8A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA7881B-2AB6-4EB5-93CA-E08E0EA8D2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DCCE98E3-7ECB-464D-B3A9-333AAEFCC845}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="79">
   <si>
     <t>substance</t>
   </si>
@@ -156,9 +156,6 @@
     <t>nom</t>
   </si>
   <si>
-    <t>Fatty acids, C7-18 and C18-unsatd., potassium salts</t>
-  </si>
-  <si>
     <t>Salmo gairdnerii</t>
   </si>
   <si>
@@ -223,6 +220,60 @@
   </si>
   <si>
     <t>Not considered in the RAR from 2023</t>
+  </si>
+  <si>
+    <t>NEU 1128 I SL</t>
+  </si>
+  <si>
+    <t>&gt;</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>RAR LoEP</t>
+  </si>
+  <si>
+    <t>Neudosan Neu Blattlausfrei</t>
+  </si>
+  <si>
+    <t>35 d</t>
+  </si>
+  <si>
+    <t>early life stage</t>
+  </si>
+  <si>
+    <t>Fatty acids C14-C20 potassium salts (ABP-617)</t>
+  </si>
+  <si>
+    <t>gmm</t>
+  </si>
+  <si>
+    <t>Chironomus riparius</t>
+  </si>
+  <si>
+    <t>ABP-617</t>
+  </si>
+  <si>
+    <t>Pseudokirchneriella subcapitata</t>
+  </si>
+  <si>
+    <t>yield</t>
+  </si>
+  <si>
+    <t>Composition</t>
+  </si>
+  <si>
+    <t>C9, i.e. the herbicidal pelargonic acid is main component, which is not one of the main components mentioned in the RAR from 2022</t>
+  </si>
+  <si>
+    <t>Fatty acids C10-C20, potassium salts</t>
+  </si>
+  <si>
+    <t>Fatty_acids_potassium_salts_RAR_33_LoEP_2022-12-21</t>
   </si>
 </sst>
 </file>
@@ -609,19 +660,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CA08FB3-CDA8-4307-B6A0-0CD6CA31604F}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" customWidth="1"/>
     <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" customWidth="1"/>
     <col min="6" max="6" width="12.140625" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" customWidth="1"/>
-    <col min="10" max="10" width="17.140625" customWidth="1"/>
-    <col min="12" max="12" width="6.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="7" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" customWidth="1"/>
+    <col min="11" max="11" width="8.42578125" customWidth="1"/>
+    <col min="12" max="12" width="4.42578125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="8.7109375" customWidth="1"/>
     <col min="14" max="14" width="7.42578125" customWidth="1"/>
     <col min="15" max="15" width="6.5703125" customWidth="1"/>
     <col min="16" max="16" width="16.42578125" customWidth="1"/>
@@ -630,7 +684,7 @@
     <col min="19" max="19" width="6.85546875" customWidth="1"/>
     <col min="20" max="20" width="7.85546875" customWidth="1"/>
     <col min="21" max="21" width="9.85546875" customWidth="1"/>
-    <col min="22" max="22" width="35.140625" customWidth="1"/>
+    <col min="22" max="22" width="30.5703125" customWidth="1"/>
     <col min="23" max="23" width="7" customWidth="1"/>
     <col min="24" max="24" width="6.85546875" customWidth="1"/>
   </cols>
@@ -709,15 +763,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -735,20 +789,22 @@
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L2" s="3"/>
+        <v>40</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M2" s="2">
         <v>8.7899999999999991</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q2" s="2">
         <v>51</v>
@@ -763,18 +819,18 @@
       </c>
       <c r="V2" s="3"/>
       <c r="W2" t="s">
+        <v>55</v>
+      </c>
+      <c r="X2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="X2" s="3" t="s">
-        <v>57</v>
-      </c>
     </row>
-    <row r="3" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>32</v>
@@ -783,11 +839,11 @@
         <v>2</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
@@ -797,18 +853,20 @@
       <c r="K3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="3"/>
+      <c r="L3" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M3" s="2">
         <v>5</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q3" s="2">
         <v>51</v>
@@ -823,19 +881,19 @@
       </c>
       <c r="V3" s="3"/>
       <c r="W3" t="s">
+        <v>55</v>
+      </c>
+      <c r="X3" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="X3" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -855,18 +913,20 @@
       <c r="K4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="3"/>
+      <c r="L4" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M4" s="2">
         <v>2</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q4" s="2">
         <v>51</v>
@@ -874,28 +934,28 @@
       <c r="R4" s="3"/>
       <c r="S4" s="2"/>
       <c r="T4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="U4" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="U4" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="V4" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="W4" t="s">
+        <v>55</v>
+      </c>
+      <c r="X4" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="X4" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D5" s="2">
         <v>3</v>
@@ -915,18 +975,20 @@
       <c r="K5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="3"/>
+      <c r="L5" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M5" s="2">
         <v>6.4</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q5" s="2">
         <v>51</v>
@@ -934,27 +996,25 @@
       <c r="R5" s="3"/>
       <c r="S5" s="2"/>
       <c r="T5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="U5" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="U5" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="V5" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="W5" t="s">
+        <v>55</v>
+      </c>
+      <c r="X5" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="X5" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>39</v>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>25</v>
@@ -977,18 +1037,20 @@
       <c r="K6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="3"/>
+      <c r="L6" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M6" s="2">
         <v>10.199999999999999</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q6" s="2">
         <v>51</v>
@@ -996,25 +1058,27 @@
       <c r="R6" s="3"/>
       <c r="S6" s="2"/>
       <c r="T6" s="3" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="U6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V6" s="3"/>
+        <v>75</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="W6" t="s">
+        <v>55</v>
+      </c>
+      <c r="X6" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="X6" s="3" t="s">
-        <v>57</v>
-      </c>
     </row>
-    <row r="7" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>25</v>
@@ -1023,32 +1087,34 @@
         <v>5</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="3"/>
+      <c r="L7" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M7" s="2">
         <v>0.5</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q7" s="2">
         <v>51</v>
@@ -1062,24 +1128,24 @@
         <v>31</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="W7" t="s">
+        <v>55</v>
+      </c>
+      <c r="X7" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="X7" s="3" t="s">
-        <v>57</v>
-      </c>
     </row>
-    <row r="8" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="2">
         <v>6</v>
@@ -1089,28 +1155,30 @@
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="3"/>
+      <c r="L8" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="M8" s="2">
         <v>1.2</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q8" s="2">
         <v>52</v>
@@ -1125,21 +1193,21 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" t="s">
+        <v>55</v>
+      </c>
+      <c r="X8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="X8" s="3" t="s">
-        <v>57</v>
-      </c>
     </row>
-    <row r="9" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="2">
         <v>6</v>
@@ -1149,7 +1217,7 @@
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3" t="s">
@@ -1164,13 +1232,13 @@
         <v>3.8</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>38</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q9" s="2">
         <v>52</v>
@@ -1185,35 +1253,554 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" t="s">
+        <v>55</v>
+      </c>
+      <c r="X9" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="X9" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" t="s">
+        <v>40</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="M10">
+        <v>37.32</v>
+      </c>
+      <c r="N10" t="s">
+        <v>41</v>
+      </c>
+      <c r="O10" t="s">
+        <v>63</v>
+      </c>
+      <c r="P10" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q10">
+        <v>96</v>
+      </c>
+      <c r="R10" t="s">
+        <v>78</v>
+      </c>
+      <c r="S10">
+        <v>96</v>
+      </c>
+      <c r="T10" t="s">
+        <v>30</v>
+      </c>
+      <c r="U10" t="s">
+        <v>65</v>
+      </c>
+      <c r="W10" t="s">
+        <v>55</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" t="s">
+        <v>68</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" t="s">
+        <v>64</v>
+      </c>
+      <c r="M11">
+        <v>1.34</v>
+      </c>
+      <c r="N11" t="s">
+        <v>41</v>
+      </c>
+      <c r="O11" t="s">
+        <v>63</v>
+      </c>
+      <c r="P11" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q11">
+        <v>97</v>
+      </c>
+      <c r="R11" t="s">
+        <v>78</v>
+      </c>
+      <c r="S11">
+        <v>97</v>
+      </c>
+      <c r="T11" t="s">
+        <v>30</v>
+      </c>
+      <c r="U11" t="s">
+        <v>65</v>
+      </c>
+      <c r="W11" t="s">
+        <v>55</v>
+      </c>
+      <c r="X11" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" t="s">
+        <v>36</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" t="s">
+        <v>64</v>
+      </c>
+      <c r="M12">
+        <v>21.6</v>
+      </c>
+      <c r="N12" t="s">
+        <v>41</v>
+      </c>
+      <c r="O12" t="s">
+        <v>63</v>
+      </c>
+      <c r="P12" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q12">
+        <v>97</v>
+      </c>
+      <c r="R12" t="s">
+        <v>78</v>
+      </c>
+      <c r="S12">
+        <v>97</v>
+      </c>
+      <c r="T12" t="s">
+        <v>30</v>
+      </c>
+      <c r="U12" t="s">
+        <v>65</v>
+      </c>
+      <c r="W12" t="s">
+        <v>55</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" t="s">
+        <v>64</v>
+      </c>
+      <c r="M13">
+        <v>0.87</v>
+      </c>
+      <c r="N13" t="s">
+        <v>41</v>
+      </c>
+      <c r="O13" t="s">
+        <v>70</v>
+      </c>
+      <c r="P13" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q13">
+        <v>97</v>
+      </c>
+      <c r="R13" t="s">
+        <v>78</v>
+      </c>
+      <c r="S13">
+        <v>97</v>
+      </c>
+      <c r="T13" t="s">
+        <v>30</v>
+      </c>
+      <c r="U13" t="s">
+        <v>65</v>
+      </c>
+      <c r="W13" t="s">
+        <v>55</v>
+      </c>
+      <c r="X13" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" t="s">
+        <v>36</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" t="s">
+        <v>62</v>
+      </c>
+      <c r="M14">
+        <v>51</v>
+      </c>
+      <c r="N14" t="s">
+        <v>41</v>
+      </c>
+      <c r="O14" t="s">
+        <v>38</v>
+      </c>
+      <c r="P14" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q14">
+        <v>97</v>
+      </c>
+      <c r="R14" t="s">
+        <v>78</v>
+      </c>
+      <c r="S14">
+        <v>97</v>
+      </c>
+      <c r="T14" t="s">
+        <v>30</v>
+      </c>
+      <c r="U14" t="s">
+        <v>65</v>
+      </c>
+      <c r="W14" t="s">
+        <v>55</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" t="s">
+        <v>64</v>
+      </c>
+      <c r="M15">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="N15" t="s">
+        <v>41</v>
+      </c>
+      <c r="O15" t="s">
+        <v>38</v>
+      </c>
+      <c r="P15" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q15">
+        <v>97</v>
+      </c>
+      <c r="R15" t="s">
+        <v>78</v>
+      </c>
+      <c r="S15">
+        <v>97</v>
+      </c>
+      <c r="T15" t="s">
+        <v>30</v>
+      </c>
+      <c r="U15" t="s">
+        <v>65</v>
+      </c>
+      <c r="W15" t="s">
+        <v>55</v>
+      </c>
+      <c r="X15" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G16" t="s">
+        <v>29</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M16">
+        <v>10</v>
+      </c>
+      <c r="N16" t="s">
+        <v>41</v>
+      </c>
+      <c r="O16" t="s">
+        <v>38</v>
+      </c>
+      <c r="P16" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q16">
+        <v>97</v>
+      </c>
+      <c r="R16" t="s">
+        <v>78</v>
+      </c>
+      <c r="S16">
+        <v>97</v>
+      </c>
+      <c r="T16" t="s">
+        <v>30</v>
+      </c>
+      <c r="U16" t="s">
+        <v>65</v>
+      </c>
+      <c r="W16" t="s">
+        <v>55</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" t="s">
+        <v>51</v>
+      </c>
+      <c r="I17" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17" t="s">
+        <v>64</v>
+      </c>
+      <c r="M17">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="N17" t="s">
+        <v>41</v>
+      </c>
+      <c r="O17" t="s">
+        <v>70</v>
+      </c>
+      <c r="P17" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q17">
+        <v>97</v>
+      </c>
+      <c r="R17" t="s">
+        <v>78</v>
+      </c>
+      <c r="S17">
+        <v>97</v>
+      </c>
+      <c r="T17" t="s">
+        <v>30</v>
+      </c>
+      <c r="U17" t="s">
+        <v>65</v>
+      </c>
+      <c r="W17" t="s">
+        <v>55</v>
+      </c>
+      <c r="X17" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18">
+        <v>14</v>
+      </c>
+      <c r="E18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" t="s">
+        <v>74</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L18" t="s">
+        <v>64</v>
+      </c>
+      <c r="M18">
+        <v>0.73</v>
+      </c>
+      <c r="N18" t="s">
+        <v>41</v>
+      </c>
+      <c r="O18" t="s">
+        <v>70</v>
+      </c>
+      <c r="P18" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q18">
+        <v>97</v>
+      </c>
+      <c r="R18" t="s">
+        <v>78</v>
+      </c>
+      <c r="S18">
+        <v>97</v>
+      </c>
+      <c r="T18" t="s">
+        <v>30</v>
+      </c>
+      <c r="U18" t="s">
+        <v>65</v>
+      </c>
+      <c r="W18" t="s">
+        <v>55</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>